<commit_message>
Visor: más polígonos y menos 'pelotitas' — preferir feature con geometría y dibujar servidumbres como línea
- bsj/cruce.py: al matchear por expediente, cuando varios features del catastro
  comparten el mismo expediente, elegir el que tiene POLÍGONO dibujable (no el
  registro Punto de la capa 'lem'). Corrige casos como 1124-108-G-22, que salían
  como punto teniendo polígono real en 'manifestaciones'.
- bsj/cruce.py: capturar también geometría LINEAL (_linea) -> linea_wgs84 en el
  bloque catastro. Las servidumbres son corredores, no áreas.
- visor.html: dibujar servidumbres como POLILÍNEA; el punto sólo queda como último
  recurso y únicamente si la ubicación es confiable (centroide del catastro). El
  centroide del boletín cuando el OCR quedó corrupto ya no se dibuja (caería mal
  ubicado). Resultado del render: 804 polígonos + 5 líneas + 1 punto (un edicto sin
  nº de expediente), contra las varias 'pelotitas' anteriores.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out_hist/pedimentos.xlsx
+++ b/out_hist/pedimentos.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N836"/>
+  <dimension ref="A1:N837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -43736,23 +43736,23 @@
     <row r="836">
       <c r="A836" t="inlineStr">
         <is>
-          <t>583-R-95</t>
+          <t>1124-242-H-13</t>
         </is>
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>Darío Becerra, Paz Eric Martín</t>
+          <t>Moncho Juan Jose y Alonso manuel Domingo</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
         <is>
-          <t>LOS CRISOLES 3</t>
+          <t>MARTINA</t>
         </is>
       </c>
       <c r="D836" t="inlineStr"/>
       <c r="E836" t="inlineStr">
         <is>
-          <t>Iglesia</t>
+          <t>Calingasta</t>
         </is>
       </c>
       <c r="F836" t="inlineStr">
@@ -43762,11 +43762,11 @@
       </c>
       <c r="G836" t="inlineStr">
         <is>
-          <t>Edicto de mensura (x3)</t>
+          <t>Edicto de mensura (x1)</t>
         </is>
       </c>
       <c r="H836" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I836" t="inlineStr">
         <is>
@@ -43777,12 +43777,67 @@
         <v>5</v>
       </c>
       <c r="L836" t="n">
+        <v>-31.096375</v>
+      </c>
+      <c r="M836" t="n">
+        <v>-69.73417999999999</v>
+      </c>
+      <c r="N836" t="inlineStr">
+        <is>
+          <t>posgar2007</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>583-R-95</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Darío Becerra, Paz Eric Martín</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>LOS CRISOLES 3</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr"/>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Iglesia</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>Edicto de mensura</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>Edicto de mensura (x3)</t>
+        </is>
+      </c>
+      <c r="H837" t="n">
+        <v>3</v>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K837" t="n">
+        <v>5</v>
+      </c>
+      <c r="L837" t="n">
         <v>-29.760661</v>
       </c>
-      <c r="M836" t="n">
+      <c r="M837" t="n">
         <v>-69.67442699999999</v>
       </c>
-      <c r="N836" t="inlineStr">
+      <c r="N837" t="inlineStr">
         <is>
           <t>posgar2007</t>
         </is>

</xml_diff>